<commit_message>
Add product names, GPT Live voice pricing and 4 full prototype units to budget
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent_sessions/2026_09_29_BREAKOUT_BARECHIP_BUDGET/Hivemind_Hardware_Budget.xlsx
+++ b/agent_sessions/2026_09_29_BREAKOUT_BARECHIP_BUDGET/Hivemind_Hardware_Budget.xlsx
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -114,10 +114,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +138,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,174 +229,19 @@
     <author>budget</author>
   </authors>
   <commentList>
-    <comment ref="A3" authorId="0" shapeId="0">
-      <text>
-        <t>nRF9151 DK (NRF9151-DK)</t>
-      </text>
-    </comment>
-    <comment ref="A4" authorId="0" shapeId="0">
-      <text>
-        <t>nRF54LM20 DK (nRF54LM20A/B, Axon enabled) (NRF54LM20-DK)</t>
-      </text>
-    </comment>
-    <comment ref="A5" authorId="0" shapeId="0">
-      <text>
-        <t>nRF7002 EK (Arduino shield) (NRF7002-EK)</t>
-      </text>
-    </comment>
-    <comment ref="A6" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit SPI Flash SD Card - XTSD 2 GB (SD NAND breakout) (6038)</t>
-      </text>
-    </comment>
-    <comment ref="A7" authorId="0" shapeId="0">
-      <text>
-        <t>Arducam Mini 2MP (OV2640, SPI + frame buffer) (B0067)</t>
-      </text>
-    </comment>
-    <comment ref="A8" authorId="0" shapeId="0">
-      <text>
-        <t>SparkFun 6DoF IMU BMI270 (Qwiic) (SEN-22397)</t>
-      </text>
-    </comment>
-    <comment ref="A9" authorId="0" shapeId="0">
-      <text>
-        <t>Waveshare UART Fingerprint Sensor (D), round capacitive (UART Fingerprint Sensor (D))</t>
-      </text>
-    </comment>
-    <comment ref="A10" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit Universal Qi Receiver Module (1901)</t>
-      </text>
-    </comment>
-    <comment ref="A11" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit Micro-Lipo Charger USB-C (4410)</t>
-      </text>
-    </comment>
-    <comment ref="A12" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit MAX17048 fuel gauge (5580)</t>
-      </text>
-    </comment>
-    <comment ref="A13" authorId="0" shapeId="0">
-      <text>
-        <t>Nordic nPM1304 EK (NPM1304-EK)</t>
-      </text>
-    </comment>
-    <comment ref="A14" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit LiPo 3.7 V 350 mAh (protected) (2750)</t>
-      </text>
-    </comment>
-    <comment ref="A15" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit DRV2605L haptic driver (2305)</t>
-      </text>
-    </comment>
-    <comment ref="A16" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit piezo buzzer PS1240 (160)</t>
-      </text>
-    </comment>
-    <comment ref="A17" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit PDM MEMS mic breakout (3492)</t>
-      </text>
-    </comment>
-    <comment ref="A18" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit MAX98357A I2S amp (3006)</t>
-      </text>
-    </comment>
-    <comment ref="A19" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit mini oval speaker 8 ohm 1 W (3923)</t>
-      </text>
-    </comment>
-    <comment ref="A20" authorId="0" shapeId="0">
-      <text>
-        <t>Waveshare 2.9in e-Paper module (296x128) (E029A01-FPCA)</t>
-      </text>
-    </comment>
-    <comment ref="A21" authorId="0" shapeId="0">
-      <text>
-        <t>Adafruit AT42QT1070 5-pad standalone (1362)</t>
-      </text>
-    </comment>
-    <comment ref="A22" authorId="0" shapeId="0">
-      <text>
-        <t>Waveshare 2.9in capacitive-touch e-Paper (Pico) (Pico-CapTouch-ePaper-2.9)</t>
-      </text>
-    </comment>
-    <comment ref="A23" authorId="0" shapeId="0">
-      <text>
-        <t>3D-printed pendant shells (JLC3DP SLA/MJF or UW DI Lab SLS), 3 iterations x 5</t>
-      </text>
-    </comment>
-    <comment ref="A24" authorId="0" shapeId="0">
-      <text>
-        <t>CNC aluminum shell samples (JLCCNC/PCBWay/Xometry), 3 pcs</t>
-      </text>
-    </comment>
-    <comment ref="A25" authorId="0" shapeId="0">
-      <text>
-        <t>Watch-band / strap samples</t>
-      </text>
-    </comment>
-    <comment ref="A26" authorId="0" shapeId="0">
-      <text>
-        <t>Necklace cord (30-pk) + breakaway clasps (50-pk) samples</t>
-      </text>
-    </comment>
-    <comment ref="A28" authorId="0" shapeId="0">
-      <text>
-        <t>Breadboards, full-size 830 tie-point</t>
-      </text>
-    </comment>
-    <comment ref="A29" authorId="0" shapeId="0">
-      <text>
-        <t>Jumper wires, premium M/M 40x150mm</t>
-      </text>
-    </comment>
     <comment ref="A30" authorId="0" shapeId="0">
       <text>
-        <t>$200/month plan (e.g. Claude Max 20x). Units = months.</t>
-      </text>
-    </comment>
-    <comment ref="A31" authorId="0" shapeId="0">
-      <text>
-        <t>KiCad (PCB design)</t>
-      </text>
-    </comment>
-    <comment ref="A32" authorId="0" shapeId="0">
-      <text>
-        <t>Onshape Education</t>
+        <t>Units = months.</t>
       </text>
     </comment>
     <comment ref="A33" authorId="0" shapeId="0">
       <text>
-        <t>OpenAI gpt-realtime-2.1-mini test audio (5,000 min)</t>
+        <t>Units = minutes of testing.</t>
       </text>
     </comment>
     <comment ref="A34" authorId="0" shapeId="0">
       <text>
-        <t>Per spin (JLCPCB 4-layer): fab + assembly fees + stencil + shipping/tariff + 3 populated boards at the per-device component cost. Units = spins.</t>
-      </text>
-    </comment>
-    <comment ref="A36" authorId="0" shapeId="0">
-      <text>
-        <t>Pinecil V2 soldering iron</t>
-      </text>
-    </comment>
-    <comment ref="A37" authorId="0" shapeId="0">
-      <text>
-        <t>Stereo/digital soldering microscope (Andonstar AD407 class)</t>
-      </text>
-    </comment>
-    <comment ref="A38" authorId="0" shapeId="0">
-      <text>
-        <t>Helping hands with 4x magnifier / PCB holder</t>
+        <t>Rough per-unit allowance. Each unit may use a different low-power chip / configuration.</t>
       </text>
     </comment>
   </commentList>
@@ -727,14 +575,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -760,6 +609,11 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>Product Name</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>Actual Product Price</t>
         </is>
       </c>
@@ -774,6 +628,7 @@
       <c r="C2" s="4" t="n"/>
       <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -792,7 +647,12 @@
           <t>digikey.com</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>nRF9151 DK</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n">
         <v>102.43</v>
       </c>
     </row>
@@ -813,7 +673,12 @@
           <t>digikey.com</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>nRF54LM20 DK</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n">
         <v>45</v>
       </c>
     </row>
@@ -834,7 +699,12 @@
           <t>digikey.com</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>nRF7002 EK</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>20.33</v>
       </c>
     </row>
@@ -855,7 +725,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit SPI Flash SD Card - XTSD 2 GB</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -874,7 +749,12 @@
           <t>uctronics.com</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Arducam Mini 2MP</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
         <v>25.99</v>
       </c>
     </row>
@@ -895,7 +775,12 @@
           <t>sparkfun.com</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>SparkFun 6DoF IMU BMI270</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
         <v>18.5</v>
       </c>
     </row>
@@ -916,7 +801,12 @@
           <t>waveshare.com</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Waveshare UART Fingerprint Sensor</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
         <v>16.99</v>
       </c>
     </row>
@@ -937,7 +827,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit Universal Qi Receiver Module</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
         <v>14.95</v>
       </c>
     </row>
@@ -958,7 +853,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit Micro-Lipo Charger USB-C</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
         <v>5.95</v>
       </c>
     </row>
@@ -979,7 +879,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit MAX17048 fuel gauge</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
         <v>5.95</v>
       </c>
     </row>
@@ -1000,7 +905,12 @@
           <t>digikey.com</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Nordic nPM1304 EK</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
         <v>46.38</v>
       </c>
     </row>
@@ -1021,7 +931,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit LiPo 3.7 V 350 mAh</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
         <v>6.95</v>
       </c>
     </row>
@@ -1042,7 +957,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit DRV2605L haptic driver</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n">
         <v>7.95</v>
       </c>
     </row>
@@ -1063,7 +983,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit piezo buzzer PS1240</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
         <v>1.5</v>
       </c>
     </row>
@@ -1084,7 +1009,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n">
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit PDM MEMS mic breakout</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n">
         <v>4.95</v>
       </c>
     </row>
@@ -1105,7 +1035,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit MAX98357A I2S amp</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>5.95</v>
       </c>
     </row>
@@ -1126,7 +1061,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit mini oval speaker 8 ohm 1 W</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1145,7 +1085,12 @@
           <t>waveshare.com</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Waveshare 2.9in e-Paper module</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>21.99</v>
       </c>
     </row>
@@ -1166,7 +1111,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n">
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Adafruit AT42QT1070 5-pad standalone</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n">
         <v>7.5</v>
       </c>
     </row>
@@ -1187,7 +1137,12 @@
           <t>waveshare.com</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n">
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Waveshare 2.9in capacitive-touch e-Paper</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
         <v>24.99</v>
       </c>
     </row>
@@ -1208,7 +1163,12 @@
           <t>jlc3dp.com</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>3D-printed pendant shells</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1227,7 +1187,12 @@
           <t>jlccnc.com</t>
         </is>
       </c>
-      <c r="E24" s="6" t="n"/>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>CNC aluminum shell samples</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1241,8 +1206,13 @@
       <c r="C25" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="6" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Watch-band / strap samples</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1261,7 +1231,12 @@
           <t>amazon.com</t>
         </is>
       </c>
-      <c r="E26" s="6" t="n"/>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Necklace cord</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1273,6 +1248,7 @@
       <c r="C27" s="4" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1291,7 +1267,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E28" s="6" t="n">
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Breadboards</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
         <v>5.95</v>
       </c>
     </row>
@@ -1312,7 +1293,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n">
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Jumper wires</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n">
         <v>3.95</v>
       </c>
     </row>
@@ -1333,7 +1319,12 @@
           <t>claude.com</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n">
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Claude Max 20x</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1354,7 +1345,12 @@
           <t>kicad.org</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n">
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>KiCad</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1375,7 +1371,12 @@
           <t>onshape.com</t>
         </is>
       </c>
-      <c r="E32" s="6" t="n">
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>Onshape Education</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1386,7 +1387,7 @@
         </is>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="C33" s="7" t="n">
         <v>5000</v>
@@ -1396,27 +1397,38 @@
           <t>openai.com</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n"/>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>GPT Live</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Prototype PCBs</t>
-        </is>
-      </c>
-      <c r="B34" s="10">
-        <f>60+86.3+16.42+45+3*'Manufacturing (30 units)'!B8</f>
-        <v/>
+          <t>Full prototype units</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>350</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
           <t>jlcpcb.com</t>
         </is>
       </c>
-      <c r="E34" s="6" t="n"/>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Complete unit: PCB + assembly + parts + shell</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1428,6 +1440,7 @@
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1446,7 +1459,12 @@
           <t>pine64.com</t>
         </is>
       </c>
-      <c r="E36" s="6" t="n">
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>Pinecil V2 soldering iron</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
         <v>35.99</v>
       </c>
     </row>
@@ -1467,7 +1485,12 @@
           <t>andonstar.com</t>
         </is>
       </c>
-      <c r="E37" s="6" t="n"/>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Stereo/digital soldering microscope</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -1486,7 +1509,12 @@
           <t>adafruit.com</t>
         </is>
       </c>
-      <c r="E38" s="6" t="n">
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Helping hands with 4x magnifier / PCB holder</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>6.95</v>
       </c>
     </row>
@@ -1497,12 +1525,13 @@
         </is>
       </c>
       <c r="B40" s="12">
-        <f>SUMPRODUCT(C2:C38,B2:B38)+SUMPRODUCT(C2:C38,(E2:E38&lt;&gt;"")*(E2:E38-B2:B38))</f>
+        <f>SUMPRODUCT(C2:C38,B2:B38)+SUMPRODUCT(C2:C38,(F2:F38&lt;&gt;"")*(F2:F38-B2:B38))</f>
         <v/>
       </c>
       <c r="C40" s="13" t="n"/>
       <c r="D40" s="13" t="n"/>
       <c r="E40" s="13" t="n"/>
+      <c r="F40" s="13" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1639,7 +1668,7 @@
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="19">
         <f>B6*C6</f>
         <v/>
       </c>
@@ -1661,7 +1690,7 @@
       <c r="C7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="19">
         <f>B7*C7</f>
         <v/>
       </c>
@@ -1677,7 +1706,7 @@
           <t>Components per device</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="19">
         <f>3.5*1+3.17*1+1.81*1+6.58*1+1.38*1+5.64*1+3.22*2+2.56*1+4.46*1+1.21*1+1.64*1+0.699*1+2.5*1+0.3*3+5.81*1+4.49*1+17.92*1+9</f>
         <v/>
       </c>
@@ -1685,7 +1714,7 @@
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="19">
         <f>B8*C8</f>
         <v/>
       </c>
@@ -1708,7 +1737,7 @@
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="19">
         <f>B9*C9</f>
         <v/>
       </c>
@@ -1731,7 +1760,7 @@
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="19">
         <f>B10*C10</f>
         <v/>
       </c>
@@ -1754,7 +1783,7 @@
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="19">
         <f>B11*C11</f>
         <v/>
       </c>
@@ -1777,7 +1806,7 @@
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="19">
         <f>B12*C12</f>
         <v/>
       </c>
@@ -1799,7 +1828,7 @@
       <c r="C13" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="19">
         <f>B13*C13</f>
         <v/>
       </c>
@@ -1815,14 +1844,14 @@
           <t>SIM + data plan, magnet, test fixture</t>
         </is>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="19">
         <f>1*$C$2+14*$C$3+1.5*$C$2+100</f>
         <v/>
       </c>
       <c r="C14" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="19">
         <f>B14*C14</f>
         <v/>
       </c>
@@ -1833,18 +1862,18 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="21">
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="22">
         <f>SUM(D6:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="20" t="n"/>
+      <c r="E15" s="21" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1852,14 +1881,14 @@
           <t>Contingency</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="23" t="n">
         <v>0.05</v>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="19">
         <f>B16*D15</f>
         <v/>
       </c>
-      <c r="E16" s="23" t="inlineStr">
+      <c r="E16" s="24" t="inlineStr">
         <is>
           <t>Of subtotal</t>
         </is>
@@ -1880,18 +1909,18 @@
       <c r="E17" s="13" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>Cost per device</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="25">
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="26">
         <f>D17/$C$3</f>
         <v/>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="27">
         <f>IF(D18&lt;=B4,"✓ Under the $"&amp;TEXT(B4,"0")&amp;" target","✗ Over the $"&amp;TEXT(B4,"0")&amp;" target")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add shared headroom runway so both budget sheets total $11,000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent_sessions/2026_09_29_BREAKOUT_BARECHIP_BUDGET/Hivemind_Hardware_Budget.xlsx
+++ b/agent_sessions/2026_09_29_BREAKOUT_BARECHIP_BUDGET/Hivemind_Hardware_Budget.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -96,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -120,6 +121,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,11 +143,10 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -575,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -640,7 +644,7 @@
         <v>102.43</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
@@ -1519,19 +1523,55 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>Total (Actual where verified, else Estimate)</t>
-        </is>
-      </c>
-      <c r="B40" s="12">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Subtotal (Actual where verified, else Estimate)</t>
+        </is>
+      </c>
+      <c r="B40" s="11">
         <f>SUMPRODUCT(C2:C38,B2:B38)+SUMPRODUCT(C2:C38,(F2:F38&lt;&gt;"")*(F2:F38-B2:B38))</f>
         <v/>
       </c>
-      <c r="C40" s="13" t="n"/>
-      <c r="D40" s="13" t="n"/>
-      <c r="E40" s="13" t="n"/>
-      <c r="F40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Headroom runway (same % on both sheets)</t>
+        </is>
+      </c>
+      <c r="B41" s="11">
+        <f>C41*B40</f>
+        <v/>
+      </c>
+      <c r="C41" s="12">
+        <f>B44/(B40+'Manufacturing (30 units)'!D15)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B42" s="14">
+        <f>B40+B41</f>
+        <v/>
+      </c>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Funding request (both sheets)</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="n">
+        <v>11000</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1592,27 +1632,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Unit Cost</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1624,10 +1664,10 @@
           <t>Board starts</t>
         </is>
       </c>
-      <c r="C2" s="16" t="n">
+      <c r="C2" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="E2" s="17" t="inlineStr">
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>30 accepted + 6 spare for yield</t>
         </is>
@@ -1639,10 +1679,10 @@
           <t>Accepted devices</t>
         </is>
       </c>
-      <c r="C3" s="16" t="n">
+      <c r="C3" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="E3" s="17" t="inlineStr"/>
+      <c r="E3" s="19" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1653,7 +1693,7 @@
       <c r="B4" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="E4" s="17" t="inlineStr"/>
+      <c r="E4" s="19" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1664,15 +1704,15 @@
       <c r="B6" s="6" t="n">
         <v>4.17</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="20">
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="11">
         <f>B6*C6</f>
         <v/>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>Derived, not quoted</t>
         </is>
@@ -1687,14 +1727,14 @@
       <c r="B7" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="11">
         <f>B7*C7</f>
         <v/>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>Setup, stencil, feeders, X-ray; not quoted</t>
         </is>
@@ -1706,19 +1746,19 @@
           <t>Components per device</t>
         </is>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="11">
         <f>3.5*1+3.17*1+1.81*1+6.58*1+1.38*1+5.64*1+3.22*2+2.56*1+4.46*1+1.21*1+1.64*1+0.699*1+2.5*1+0.3*3+5.81*1+4.49*1+17.92*1+9</f>
         <v/>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="20">
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="11">
         <f>B8*C8</f>
         <v/>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>Core bare chips at qty-100 + $9 passives allowance</t>
         </is>
@@ -1733,15 +1773,15 @@
       <c r="B9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="20">
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="11">
         <f>B9*C9</f>
         <v/>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>CNC aluminum would break the target</t>
         </is>
@@ -1756,15 +1796,15 @@
       <c r="B10" s="6" t="n">
         <v>2.5</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="20">
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="11">
         <f>B10*C10</f>
         <v/>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>Cord with breakaway clasp</t>
         </is>
@@ -1779,15 +1819,15 @@
       <c r="B11" s="6" t="n">
         <v>4.46</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="20">
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="11">
         <f>B11*C11</f>
         <v/>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>$4.46 at 10+ (Adafruit)</t>
         </is>
@@ -1802,15 +1842,15 @@
       <c r="B12" s="6" t="n">
         <v>2.5</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="20">
         <f>$C$2</f>
         <v/>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="11">
         <f>B12*C12</f>
         <v/>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>Box, foam, card</t>
         </is>
@@ -1825,14 +1865,14 @@
       <c r="B13" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="11">
         <f>B13*C13</f>
         <v/>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>JLCPCB DHL + US DDP tariff, DigiKey freight</t>
         </is>
@@ -1844,83 +1884,84 @@
           <t>SIM + data plan, magnet, test fixture</t>
         </is>
       </c>
-      <c r="B14" s="19">
+      <c r="B14" s="11">
         <f>1*$C$2+14*$C$3+1.5*$C$2+100</f>
         <v/>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="11">
         <f>B14*C14</f>
         <v/>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>1NCE $1 SIM x starts + $14 plan x accepted; magnet; pogo jig</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="22">
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="23">
         <f>SUM(D6:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="21" t="n"/>
+      <c r="E15" s="22" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B16" s="23" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D16" s="19">
+          <t>Headroom runway (same % on both sheets)</t>
+        </is>
+      </c>
+      <c r="B16" s="24">
+        <f>Components!C41</f>
+        <v/>
+      </c>
+      <c r="D16" s="11">
         <f>B16*D15</f>
         <v/>
       </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>Of subtotal</t>
+      <c r="E16" s="25" t="inlineStr">
+        <is>
+          <t>Both sheets together = funding request</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="12">
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="14">
         <f>D15+D16</f>
         <v/>
       </c>
-      <c r="E17" s="13" t="n"/>
+      <c r="E17" s="15" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>Cost per device</t>
         </is>
       </c>
-      <c r="B18" s="21" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="26">
+      <c r="B18" s="22" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="27">
         <f>D17/$C$3</f>
         <v/>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="28">
         <f>IF(D18&lt;=B4,"✓ Under the $"&amp;TEXT(B4,"0")&amp;" target","✗ Over the $"&amp;TEXT(B4,"0")&amp;" target")</f>
         <v/>
       </c>

</xml_diff>